<commit_message>
feat(standards): enforce serialized naming conventions and resolve 404 on relative document paths
- Enforce standard serialization across docs/ (00_AUTONOMOUS_OPTIMIZATION_LOOP.md, 01_METHODOLOGY_AND_CONTEXT_MEMORY.md, 02_PROJECT_PLAN_AND_CONVENTIONS.xlsx, 03_GLOBAL_LOCK_DATA_INDEX.xlsx, 04_GALLERY_STYLE_RESTRUCTURING_GUIDE.md)
- Update tools/generate-project-excel.py and tools/generate-master-index-excel.py to generate indexed sheets and files
- Fix serve.mjs routing for relative /zh/docs/ and /en/docs/ requests resolving 404 to HTTP 200 OK
- 23 scoring + 36 site integrity tests pass 100%

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/GLOBAL_LOCK_DATA_INDEX.xlsx
+++ b/docs/GLOBAL_LOCK_DATA_INDEX.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全局数据资产索引总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="日本面板刻印反查索引" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="转接件BOM与公差索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="开孔打样工程模板索引" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="海外爆款机械锁兼容索引" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="真实故障避坑工单索引" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="01_全局数据资产索引总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_日本面板刻印反查索引" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03_转接件BOM与公差索引" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04_开孔打样工程模板索引" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05_海外爆款机械锁兼容索引" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="06_真实故障避坑工单索引" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,22 +477,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="43" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 全局数据资产索引总览</t>
+          <t>GlobalLockSummary 全局索引 — 01_全局数据资产索引总览</t>
         </is>
       </c>
     </row>
@@ -500,35 +501,40 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>模块序号</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>模块大类</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>数据分类 / 业务主题</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>涵盖记录数</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>物理存储文件</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>在线访问页面</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>关联抓取实物图路径</t>
-        </is>
-      </c>
       <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>关联实物图路径</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>核心作用与工程价值</t>
         </is>
@@ -537,146 +543,166 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>IDX-01</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>1. 工业板块与图墙</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>5大标准板块与32类实物图谱</t>
-        </is>
-      </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>32 种锁型</t>
+          <t>5大标准板块与38类实物图谱</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>38 种锁型</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
           <t>content/catalog/gallery.json</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>/zh/index.html</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>assets/img/gallery/*_real.jpg</t>
-        </is>
-      </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>全球存量锁真实安装实景，按 ASSA ABLOY 分区与动态计数直观呈现</t>
+          <t>assets/img/gallery/*_real.*</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>全球存量锁真实安装实景，按 ASSA ABLOY 分区与动态计数呈现</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>IDX-02</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
           <t>1. 工业板块与图墙</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>3大强相关基准锁 Block-Hero</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>3 款基准</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>assets/img/hero/*.jpg</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>/zh/index.html 展板</t>
-        </is>
-      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
+          <t>/zh/index.html</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>assets/img/hero/hero-*.jpg</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>北美 Deadbolt、欧标双锁芯、澳式 001 顶级入口超大图与死穴直达</t>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>北美 Deadbolt、欧标双锁芯、澳式 001 顶级大主图入口</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>IDX-03</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
           <t>2. 本土辨锁大百科</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>5国本土语言测锁与工业术语</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>5 大国别体系</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>content/catalog/indigenous-lock-guides.json</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>/zh/indigenous-guides.html</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>assets/img/indigenous/*.png|jpg</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>收录德、法、日、英、西本土锁匠量测口诀，破解 Dornmaß、Axe、Entraxe 差异</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>收录德、法、日、英、西本土锁匠量测口诀，破解 Dornmaß、Axe 差异</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>IDX-04</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
           <t>3. 专项研发工具</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>日本主流门锁面板刻印速查字典</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>5 大主力锁族 (28+刻印)</t>
-        </is>
-      </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
+          <t>5 大主力锁族</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
           <t>content/catalog/japan-engraving-matrix.json</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>/zh/japan-engravings.html</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>assets/img/indigenous/jp-*.jpg</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>刻印即型号，输入 MIWA/GOAL 刻印 1 秒获取 CAD 开孔与专用夹爪</t>
         </is>
@@ -685,72 +711,82 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>IDX-05</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>3. 专项研发工具</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>全球智能锁 Retrofit 标准转接件 BOM</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>4 款核心转接套</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>content/catalog/adapters-bom.json</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>/zh/adapters.html</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>assets/img/tools/adapter-7to8mm.png</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>法国 7转8mm 变径方轴、德标 8转9mm 逃生套、美标十字尾轴盘、日本捏合爪</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>法国 7转8mm 铜套、德标 8转9mm 逃生套、美标十字尾轴盘、日本捏合爪</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>IDX-06</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
           <t>3. 专项研发工具</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>海外主流防盗锁 1:1 官方开孔打样模板</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>3 套原厂规范</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>content/catalog/drilling-templates.json</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>/zh/drilling-templates.html</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>assets/img/tools/template-*.png</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>北美 ANSI 54mm 大孔、日本 42mm 螺栓距、欧标 72/92mm PZ 开孔规程</t>
         </is>
@@ -759,35 +795,40 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>IDX-07</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
           <t>4. 改装排雷与电商</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>全球智能锁改装一线避坑实录</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>4 大经典故障源</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>content/catalog/field-issues.json</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>/zh/field-issues.html</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>assets/img/tools/gap-clearance.jpg</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>抓取 Reddit / 锁匠工单真实差评：抬把手过载、门缝卡阻、离合反锁、胶贴脱落</t>
         </is>
@@ -796,35 +837,40 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>IDX-08</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
           <t>4. 改装排雷与电商</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>海外跨境爆款机械锁兼容性排行榜</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>4 国顶流爆款</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>content/catalog/bestseller-locks.json</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>/zh/bestseller-matrix.html</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>assets/img/tools/bestseller-deadbolt.jpg</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>美亚 Kwikset、德亚 ABUS、日本乐天 MIWA、英亚 Yale 畅销机械锁改装适配榜</t>
         </is>
@@ -833,35 +879,40 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>IDX-09</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>5. 核心机读数据</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>全站全量机读数据集 API</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>全部数据汇总</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>_site/data/catalog.json</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>/data/catalog.json</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>全站资产统一引用</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>供企业研发系统、移动端 App、出海选型工具直接一键 GET 拉取调用</t>
         </is>
@@ -870,35 +921,40 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>IDX-10</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
           <t>5. 核心机读数据</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>站内全文检索实时倒排索引</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>118 个页面索引</t>
-        </is>
-      </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
+          <t>128 个页面索引</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
           <t>_site/data/search-index.json</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>/search.html</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>站内全局搜索</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>全站全文分词索引，支持任意型号、术语、公差毫秒级搜索联想</t>
         </is>
@@ -915,24 +971,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="41" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="41" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 日本面板刻印反查索引</t>
+          <t>GlobalLockSummary 全局索引 — 02_日本面板刻印反查索引</t>
         </is>
       </c>
     </row>
@@ -940,45 +997,50 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>刻印编号</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>制造品牌</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>面板冲压刻印 (フロント刻印)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>机械锁具类别</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>标准背距 (Backset)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>对应门厚 (Door Thickness)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>改装难度评级</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>推荐加装智能锁 / 适配夹爪</t>
-        </is>
-      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>推荐加装智能锁</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>实物/CAD图片文件</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>关键工程死穴与要点</t>
         </is>
@@ -987,45 +1049,50 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>KOK-01</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>MIWA (美和ロック)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>LA / 13LA / LA・MA</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>插芯呆锁与把手联动锁 (Mortise Latch &amp; Deadbolt)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>51mm / 64mm</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>33 ~ 42mm</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>极易 (Very Easy)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>SwitchBot Lock Ultra (Adapter C), Sada-Elinx M-Kit, Qrio Lock Q-SL2</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>assets/img/tools/template-miwa-la.jpg</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>日本保有量最大的主力门锁。Retrofit 适配器极为成熟，需注意若为 B5 防盗旋钮，必须选择带侧按捏合爪的套件。</t>
         </is>
@@ -1034,45 +1101,50 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>KOK-02</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
           <t>MIWA (美和ロック)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>BH / DZ / LD / LDSP</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>插芯呆锁 (Mortise Deadbolt Only)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>31mm / 51mm / 64mm</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>33 ~ 42mm</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>易 (Easy)</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>SwitchBot Lock Pro, Qrio Lock</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>assets/img/indigenous/jp-thumbturn.jpg</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>常用于副锁或窄边框木门/铝合金门，旋钮间距与把手无关，直接吸附即可。</t>
         </is>
@@ -1081,45 +1153,50 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>KOK-03</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
           <t>MIWA (美和ロック)</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>LSP / LE / SWLSP / TE</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>轻型插芯锁 (Small Backset Mortise)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>51mm / 64mm</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>28 ~ 40mm</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>易 (Easy)</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>SwitchBot, Qrio, Sada</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>assets/img/indigenous/jp-thumbturn.jpg</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>集合住宅（公寓）极高频出现，锁芯通过螺纹或 U 销与锁体紧固。</t>
         </is>
@@ -1128,45 +1205,50 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>KOK-04</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
           <t>GOAL (ゴール)</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>LX / AS・LX / LG</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>高安全插芯把手锁</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>38mm / 51mm / 64mm</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>33 ~ 43mm</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>易 (Easy)</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>SwitchBot Lock Pro (Adapter G), Aqara U200</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>assets/img/indigenous/jp-miwa-13la.jpg</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>日本市场占有率仅次于 MIWA，旋钮行程一般为 90 度整，旋转阻尼适中。</t>
         </is>
@@ -1175,45 +1257,50 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>KOK-05</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>SHOWA (昭和)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>CL / 516 / 397</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>插芯逃生锁</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>50mm / 60mm</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>30 ~ 42mm</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>中等 (Moderate)</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>通用可调式机械抓爪</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>assets/img/indigenous/jp-miwa-13la.jpg</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>老式公团住宅多见，旋钮行程较长（约 105 度），需确保智能锁电机行程自学习充分。</t>
         </is>
@@ -1231,7 +1318,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
@@ -1247,7 +1334,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 转接件BOM与公差索引</t>
+          <t>GlobalLockSummary 全局索引 — 03_转接件BOM与公差索引</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1389,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>adp-fr-7to8</t>
+          <t>ADP-01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1349,7 +1436,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>adp-de-8to9</t>
+          <t>ADP-02</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1396,7 +1483,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>adp-jp-b5-gripper</t>
+          <t>ADP-03</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1443,7 +1530,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>adp-us-tailpiece-cross</t>
+          <t>ADP-04</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1499,7 +1586,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
@@ -1515,7 +1602,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 开孔打样工程模板索引</t>
+          <t>GlobalLockSummary 全局索引 — 04_开孔打样工程模板索引</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1657,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>tpl-us-ansi-deadbolt</t>
+          <t>TPL-01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1617,7 +1704,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>tpl-jp-miwa-la</t>
+          <t>TPL-02</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1664,7 +1751,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>tpl-eu-din-18251</t>
+          <t>TPL-03</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1720,7 +1807,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -1737,7 +1824,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 海外爆款机械锁兼容索引</t>
+          <t>GlobalLockSummary 全局索引 — 05_海外爆款机械锁兼容索引</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1832,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>榜单编号</t>
+          <t>爆款编号</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1797,7 +1884,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>best-us-deadbolt</t>
+          <t>BST-01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1849,7 +1936,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>best-de-abus-d6x</t>
+          <t>BST-02</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1901,7 +1988,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>best-jp-miwa-la</t>
+          <t>BST-03</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1953,7 +2040,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>best-uk-yale-nightlatch</t>
+          <t>BST-04</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2014,7 +2101,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="43" customWidth="1" min="2" max="2"/>
@@ -2030,7 +2117,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GlobalLockSummary 全局索引 — 真实故障避坑工单索引</t>
+          <t>GlobalLockSummary 全局索引 — 06_真实故障避坑工单索引</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2172,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>ISSUE-01</t>
+          <t>FL-01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -2132,7 +2219,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>ISSUE-02</t>
+          <t>FL-02</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2179,7 +2266,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ISSUE-03</t>
+          <t>FL-03</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2226,7 +2313,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ISSUE-04</t>
+          <t>FL-04</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2273,7 +2360,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ISSUE-05</t>
+          <t>FL-05</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">

</xml_diff>